<commit_message>
Corrige escrita do HTML em UTF-8 (Windows) e melhora casamento OpenAlex
- coword_analysis.py: grava a rede interativa com encoding UTF-8 explícito,
  evitando UnicodeEncodeError do pyvis no Windows (codec cp1252).
- enrich_metadata.py: avalia os 5 melhores candidatos do OpenAlex e escolhe
  o de maior similaridade de título (em vez do 1º), com limpeza de título
  mais robusta, para aumentar a cobertura do enriquecimento.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Fvrdaa5i99DsPUToDczGGv
</commit_message>
<xml_diff>
--- a/output/coword/coword_nos_comunidades.xlsx
+++ b/output/coword/coword_nos_comunidades.xlsx
@@ -441,203 +441,203 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>networks</t>
+          <t>brazilian</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>41</v>
+        <v>57</v>
       </c>
       <c r="C2" t="n">
         <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>60</v>
+        <v>69</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>neural</t>
+          <t>portuguese</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>29</v>
+        <v>50</v>
       </c>
       <c r="C3" t="n">
         <v>0</v>
       </c>
       <c r="D3" t="n">
-        <v>37</v>
+        <v>52</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>classification</t>
+          <t>speech</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C4" t="n">
         <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>23</v>
+        <v>35</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>neural networks</t>
+          <t>language</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="C5" t="n">
         <v>0</v>
       </c>
       <c r="D5" t="n">
-        <v>18</v>
+        <v>29</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>network</t>
+          <t>brazilian portuguese</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="C6" t="n">
         <v>0</v>
       </c>
       <c r="D6" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>graph</t>
+          <t>intelligent</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="C7" t="n">
         <v>0</v>
       </c>
       <c r="D7" t="n">
-        <v>19</v>
+        <v>15</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>dynamic</t>
+          <t>corpus</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="C8" t="n">
         <v>0</v>
       </c>
       <c r="D8" t="n">
-        <v>16</v>
+        <v>29</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>heterogeneous</t>
+          <t>evaluation</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="C9" t="n">
         <v>0</v>
       </c>
       <c r="D9" t="n">
-        <v>9</v>
+        <v>27</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ocean</t>
+          <t>recognition</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="C10" t="n">
         <v>0</v>
       </c>
       <c r="D10" t="n">
-        <v>15</v>
+        <v>26</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>model</t>
+          <t>automatic</t>
         </is>
       </c>
       <c r="B11" t="n">
+        <v>10</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" t="n">
         <v>9</v>
-      </c>
-      <c r="C11" t="n">
-        <v>0</v>
-      </c>
-      <c r="D11" t="n">
-        <v>12</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>embedding</t>
+          <t>resources</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C12" t="n">
         <v>0</v>
       </c>
       <c r="D12" t="n">
-        <v>13</v>
+        <v>24</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>complex</t>
+          <t>cham</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C13" t="n">
         <v>0</v>
       </c>
       <c r="D13" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>joint</t>
+          <t>natural</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C14" t="n">
         <v>0</v>
@@ -649,7 +649,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>neural network</t>
+          <t>computer</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -659,161 +659,161 @@
         <v>0</v>
       </c>
       <c r="D15" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>surface</t>
+          <t>design</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C16" t="n">
         <v>0</v>
       </c>
       <c r="D16" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ijcnn</t>
+          <t>science</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C17" t="n">
         <v>0</v>
       </c>
       <c r="D17" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>graph neural</t>
+          <t>bracis</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C18" t="n">
         <v>0</v>
       </c>
       <c r="D18" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>networks ijcnn</t>
+          <t>computational</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C19" t="n">
         <v>0</v>
       </c>
       <c r="D19" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>arctic</t>
+          <t>public</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C20" t="n">
         <v>0</v>
       </c>
       <c r="D20" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>propagation</t>
+          <t>speech recognition</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C21" t="n">
         <v>0</v>
       </c>
       <c r="D21" t="n">
-        <v>6</v>
+        <v>13</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>resilience</t>
+          <t>asr</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C22" t="n">
         <v>0</v>
       </c>
       <c r="D22" t="n">
-        <v>10</v>
+        <v>19</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>selection</t>
+          <t>online</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C23" t="n">
         <v>0</v>
       </c>
       <c r="D23" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>estimation</t>
+          <t>spontaneous</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C24" t="n">
         <v>0</v>
       </c>
       <c r="D24" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>physics-informed</t>
+          <t>applied</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C25" t="n">
         <v>0</v>
@@ -825,7 +825,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>offshore</t>
+          <t>extraction</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -835,13 +835,13 @@
         <v>0</v>
       </c>
       <c r="D26" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>assessment</t>
+          <t>development</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -851,13 +851,13 @@
         <v>0</v>
       </c>
       <c r="D27" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>physics-informed neural</t>
+          <t>natural language</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -873,23 +873,23 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>event</t>
+          <t>portuguese language</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C29" t="n">
         <v>0</v>
       </c>
       <c r="D29" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>operator</t>
+          <t>latin</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -899,13 +899,13 @@
         <v>0</v>
       </c>
       <c r="D30" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>neural operator</t>
+          <t>index</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -915,13 +915,13 @@
         <v>0</v>
       </c>
       <c r="D31" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>ocean offshore</t>
+          <t>corpora</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -931,13 +931,13 @@
         <v>0</v>
       </c>
       <c r="D32" t="n">
-        <v>6</v>
+        <v>13</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>bayesian</t>
+          <t>weather</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -947,13 +947,13 @@
         <v>0</v>
       </c>
       <c r="D33" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>eng</t>
+          <t>american</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -963,13 +963,13 @@
         <v>0</v>
       </c>
       <c r="D34" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>synchronization</t>
+          <t>probabilistic</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -979,13 +979,13 @@
         <v>0</v>
       </c>
       <c r="D35" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>fine-tuning</t>
+          <t>aspects</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1001,7 +1001,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>feature</t>
+          <t>features</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1011,13 +1011,13 @@
         <v>0</v>
       </c>
       <c r="D37" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>complex networks</t>
+          <t>insurance</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1027,13 +1027,13 @@
         <v>0</v>
       </c>
       <c r="D38" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>semi-supervised</t>
+          <t>emotion</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1043,401 +1043,401 @@
         <v>0</v>
       </c>
       <c r="D39" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>brazilian</t>
+          <t>coraa</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>57</v>
+        <v>4</v>
       </c>
       <c r="C40" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D40" t="n">
-        <v>69</v>
+        <v>12</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>portuguese</t>
+          <t>philosophy</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>50</v>
+        <v>4</v>
       </c>
       <c r="C41" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D41" t="n">
-        <v>52</v>
+        <v>6</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>speech</t>
+          <t>formal</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>23</v>
+        <v>4</v>
       </c>
       <c r="C42" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D42" t="n">
-        <v>35</v>
+        <v>12</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>language</t>
+          <t>spoken</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>22</v>
+        <v>4</v>
       </c>
       <c r="C43" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D43" t="n">
-        <v>29</v>
+        <v>11</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>brazilian portuguese</t>
+          <t>emotion recognition</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="C44" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D44" t="n">
-        <v>22</v>
+        <v>5</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>intelligent</t>
+          <t>manually</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="C45" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D45" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>corpus</t>
+          <t>data</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>18</v>
+        <v>42</v>
       </c>
       <c r="C46" t="n">
         <v>1</v>
       </c>
       <c r="D46" t="n">
-        <v>29</v>
+        <v>63</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>recognition</t>
+          <t>artificial</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="C47" t="n">
         <v>1</v>
       </c>
       <c r="D47" t="n">
-        <v>26</v>
+        <v>33</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>evaluation</t>
+          <t>intelligence</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="C48" t="n">
         <v>1</v>
       </c>
       <c r="D48" t="n">
-        <v>27</v>
+        <v>30</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>processing</t>
+          <t>artificial intelligence</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C49" t="n">
         <v>1</v>
       </c>
       <c r="D49" t="n">
-        <v>22</v>
+        <v>18</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>automatic</t>
+          <t>detection</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="C50" t="n">
         <v>1</v>
       </c>
       <c r="D50" t="n">
-        <v>9</v>
+        <v>24</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>resources</t>
+          <t>processing</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C51" t="n">
         <v>1</v>
       </c>
       <c r="D51" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>cham</t>
+          <t>engineering</t>
         </is>
       </c>
       <c r="B52" t="n">
+        <v>11</v>
+      </c>
+      <c r="C52" t="n">
+        <v>1</v>
+      </c>
+      <c r="D52" t="n">
         <v>9</v>
-      </c>
-      <c r="C52" t="n">
-        <v>1</v>
-      </c>
-      <c r="D52" t="n">
-        <v>5</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>design</t>
+          <t>inteligência</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C53" t="n">
         <v>1</v>
       </c>
       <c r="D53" t="n">
-        <v>15</v>
+        <v>6</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>bracis</t>
+          <t>inteligência artificial</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C54" t="n">
         <v>1</v>
       </c>
       <c r="D54" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>speech recognition</t>
+          <t>datasets</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C55" t="n">
         <v>1</v>
       </c>
       <c r="D55" t="n">
-        <v>13</v>
+        <v>6</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>spontaneous</t>
+          <t>news</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C56" t="n">
         <v>1</v>
       </c>
       <c r="D56" t="n">
-        <v>13</v>
+        <v>6</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>online</t>
+          <t>fair</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C57" t="n">
         <v>1</v>
       </c>
       <c r="D57" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>asr</t>
+          <t>inteligencia artificial</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C58" t="n">
         <v>1</v>
       </c>
       <c r="D58" t="n">
-        <v>19</v>
+        <v>2</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>public</t>
+          <t>agriculture</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C59" t="n">
         <v>1</v>
       </c>
       <c r="D59" t="n">
-        <v>15</v>
+        <v>5</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>portuguese language</t>
+          <t>digital</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C60" t="n">
         <v>1</v>
       </c>
       <c r="D60" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>development</t>
+          <t>inteligencia</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C61" t="n">
         <v>1</v>
       </c>
       <c r="D61" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>extraction</t>
+          <t>multimodal</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C62" t="n">
         <v>1</v>
       </c>
       <c r="D62" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>manually</t>
+          <t>regulação</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C63" t="n">
         <v>1</v>
       </c>
       <c r="D63" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>coraa</t>
+          <t>knowledge</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C64" t="n">
         <v>1</v>
@@ -1449,43 +1449,43 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>aspects</t>
+          <t>agricultural</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C65" t="n">
         <v>1</v>
       </c>
       <c r="D65" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>index</t>
+          <t>fake</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C66" t="n">
         <v>1</v>
       </c>
       <c r="D66" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>american</t>
+          <t>fake news</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C67" t="n">
         <v>1</v>
@@ -1497,238 +1497,238 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>insurance</t>
+          <t>computacional</t>
         </is>
       </c>
       <c r="B68" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C68" t="n">
         <v>1</v>
       </c>
       <c r="D68" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>corpora</t>
+          <t>data augmentation</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C69" t="n">
         <v>1</v>
       </c>
       <c r="D69" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>latin</t>
+          <t>nacional</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C70" t="n">
         <v>1</v>
       </c>
       <c r="D70" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>emotion</t>
+          <t>sul</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C71" t="n">
         <v>1</v>
       </c>
       <c r="D71" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>weather</t>
+          <t>set</t>
         </is>
       </c>
       <c r="B72" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C72" t="n">
         <v>1</v>
       </c>
       <c r="D72" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>spoken</t>
+          <t>events</t>
         </is>
       </c>
       <c r="B73" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C73" t="n">
         <v>1</v>
       </c>
       <c r="D73" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>emotion recognition</t>
+          <t>facial</t>
         </is>
       </c>
       <c r="B74" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C74" t="n">
         <v>1</v>
       </c>
       <c r="D74" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>features</t>
+          <t>augmentation</t>
         </is>
       </c>
       <c r="B75" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C75" t="n">
         <v>1</v>
       </c>
       <c r="D75" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>universal</t>
+          <t>amazon</t>
         </is>
       </c>
       <c r="B76" t="n">
-        <v>32</v>
+        <v>4</v>
       </c>
       <c r="C76" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D76" t="n">
-        <v>23</v>
+        <v>8</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>dependencies</t>
+          <t>early</t>
         </is>
       </c>
       <c r="B77" t="n">
-        <v>31</v>
+        <v>4</v>
       </c>
       <c r="C77" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D77" t="n">
-        <v>24</v>
+        <v>10</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>universal dependencies</t>
+          <t>low-resource</t>
         </is>
       </c>
       <c r="B78" t="n">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="C78" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D78" t="n">
-        <v>23</v>
+        <v>4</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>português</t>
+          <t>agricultura</t>
         </is>
       </c>
       <c r="B79" t="n">
-        <v>23</v>
+        <v>4</v>
       </c>
       <c r="C79" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D79" t="n">
-        <v>27</v>
+        <v>3</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>brasileiro</t>
+          <t>reconhecimento</t>
         </is>
       </c>
       <c r="B80" t="n">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="C80" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D80" t="n">
-        <v>15</v>
+        <v>4</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>september</t>
+          <t>data intelligence</t>
         </is>
       </c>
       <c r="B81" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="C81" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D81" t="n">
-        <v>6</v>
+        <v>14</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>brasil</t>
+          <t>build</t>
         </is>
       </c>
       <c r="B82" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C82" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D82" t="n">
         <v>10</v>
@@ -1737,494 +1737,494 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>tweets</t>
+          <t>blue amazon</t>
         </is>
       </c>
       <c r="B83" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C83" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D83" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>opinion</t>
+          <t>extrusion</t>
         </is>
       </c>
       <c r="B84" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C84" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D84" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>estudo</t>
+          <t>diagnosis</t>
         </is>
       </c>
       <c r="B85" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C85" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D85" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>portugues</t>
+          <t>building</t>
         </is>
       </c>
       <c r="B86" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C86" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D86" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>texts</t>
+          <t>agricultura digital</t>
         </is>
       </c>
       <c r="B87" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C87" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D87" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>dados</t>
+          <t>blue</t>
         </is>
       </c>
       <c r="B88" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C88" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D88" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>mercado financeiro</t>
+          <t>networks</t>
         </is>
       </c>
       <c r="B89" t="n">
-        <v>6</v>
+        <v>41</v>
       </c>
       <c r="C89" t="n">
         <v>2</v>
       </c>
       <c r="D89" t="n">
-        <v>6</v>
+        <v>60</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>mercado</t>
+          <t>neural</t>
         </is>
       </c>
       <c r="B90" t="n">
-        <v>6</v>
+        <v>29</v>
       </c>
       <c r="C90" t="n">
         <v>2</v>
       </c>
       <c r="D90" t="n">
-        <v>6</v>
+        <v>37</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>lexical</t>
+          <t>classification</t>
         </is>
       </c>
       <c r="B91" t="n">
-        <v>6</v>
+        <v>24</v>
       </c>
       <c r="C91" t="n">
         <v>2</v>
       </c>
       <c r="D91" t="n">
-        <v>4</v>
+        <v>23</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>construções</t>
+          <t>neural networks</t>
         </is>
       </c>
       <c r="B92" t="n">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="C92" t="n">
         <v>2</v>
       </c>
       <c r="D92" t="n">
-        <v>8</v>
+        <v>18</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>parsing</t>
+          <t>network</t>
         </is>
       </c>
       <c r="B93" t="n">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="C93" t="n">
         <v>2</v>
       </c>
       <c r="D93" t="n">
-        <v>10</v>
+        <v>19</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>financeiro</t>
+          <t>graph</t>
         </is>
       </c>
       <c r="B94" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="C94" t="n">
         <v>2</v>
       </c>
       <c r="D94" t="n">
-        <v>6</v>
+        <v>19</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>linguagem</t>
+          <t>ocean</t>
         </is>
       </c>
       <c r="B95" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="C95" t="n">
         <v>2</v>
       </c>
       <c r="D95" t="n">
-        <v>8</v>
+        <v>15</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>português brasileiro</t>
+          <t>model</t>
         </is>
       </c>
       <c r="B96" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="C96" t="n">
         <v>2</v>
       </c>
       <c r="D96" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>segundo</t>
+          <t>heterogeneous</t>
         </is>
       </c>
       <c r="B97" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="C97" t="n">
         <v>2</v>
       </c>
       <c r="D97" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>annotation</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="B98" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="C98" t="n">
         <v>2</v>
       </c>
       <c r="D98" t="n">
-        <v>4</v>
+        <v>16</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>informação</t>
+          <t>embedding</t>
         </is>
       </c>
       <c r="B99" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C99" t="n">
         <v>2</v>
       </c>
       <c r="D99" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>caso</t>
+          <t>joint</t>
         </is>
       </c>
       <c r="B100" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C100" t="n">
         <v>2</v>
       </c>
       <c r="D100" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>análise</t>
+          <t>complex</t>
         </is>
       </c>
       <c r="B101" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C101" t="n">
         <v>2</v>
       </c>
       <c r="D101" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>abralin</t>
+          <t>neural network</t>
         </is>
       </c>
       <c r="B102" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C102" t="n">
         <v>2</v>
       </c>
       <c r="D102" t="n">
-        <v>5</v>
+        <v>13</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>base</t>
+          <t>networks ijcnn</t>
         </is>
       </c>
       <c r="B103" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C103" t="n">
         <v>2</v>
       </c>
       <c r="D103" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>processamento</t>
+          <t>ijcnn</t>
         </is>
       </c>
       <c r="B104" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C104" t="n">
         <v>2</v>
       </c>
       <c r="D104" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>portuguese texts</t>
+          <t>surface</t>
         </is>
       </c>
       <c r="B105" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C105" t="n">
         <v>2</v>
       </c>
       <c r="D105" t="n">
-        <v>7</v>
+        <v>17</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>tweets mercado</t>
+          <t>graph neural</t>
         </is>
       </c>
       <c r="B106" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C106" t="n">
         <v>2</v>
       </c>
       <c r="D106" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>relações</t>
+          <t>assessment</t>
         </is>
       </c>
       <c r="B107" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C107" t="n">
         <v>2</v>
       </c>
       <c r="D107" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>annotated</t>
+          <t>resilience</t>
         </is>
       </c>
       <c r="B108" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C108" t="n">
         <v>2</v>
       </c>
       <c r="D108" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>artificial</t>
+          <t>estimation</t>
         </is>
       </c>
       <c r="B109" t="n">
-        <v>35</v>
+        <v>5</v>
       </c>
       <c r="C109" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D109" t="n">
-        <v>33</v>
+        <v>1</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>intelligence</t>
+          <t>arctic</t>
         </is>
       </c>
       <c r="B110" t="n">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="C110" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D110" t="n">
-        <v>30</v>
+        <v>12</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>artificial intelligence</t>
+          <t>offshore</t>
         </is>
       </c>
       <c r="B111" t="n">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="C111" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D111" t="n">
-        <v>18</v>
+        <v>12</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>optimization</t>
+          <t>selection</t>
         </is>
       </c>
       <c r="B112" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="C112" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D112" t="n">
-        <v>14</v>
+        <v>4</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>engineering</t>
+          <t>physics-informed neural</t>
         </is>
       </c>
       <c r="B113" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="C113" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D113" t="n">
         <v>9</v>
@@ -2233,14 +2233,14 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>inteligência</t>
+          <t>propagation</t>
         </is>
       </c>
       <c r="B114" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="C114" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D114" t="n">
         <v>6</v>
@@ -2249,190 +2249,190 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>inteligência artificial</t>
+          <t>physics-informed</t>
         </is>
       </c>
       <c r="B115" t="n">
+        <v>5</v>
+      </c>
+      <c r="C115" t="n">
+        <v>2</v>
+      </c>
+      <c r="D115" t="n">
         <v>9</v>
-      </c>
-      <c r="C115" t="n">
-        <v>3</v>
-      </c>
-      <c r="D115" t="n">
-        <v>6</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>news</t>
+          <t>operator</t>
         </is>
       </c>
       <c r="B116" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C116" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D116" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>inteligencia artificial</t>
+          <t>neural operator</t>
         </is>
       </c>
       <c r="B117" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C117" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D117" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>digital</t>
+          <t>eng</t>
         </is>
       </c>
       <c r="B118" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C118" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D118" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>inteligencia</t>
+          <t>synchronization</t>
         </is>
       </c>
       <c r="B119" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C119" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D119" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>regulação</t>
+          <t>semi-supervised</t>
         </is>
       </c>
       <c r="B120" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C120" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D120" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>multimodal</t>
+          <t>ocean offshore</t>
         </is>
       </c>
       <c r="B121" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C121" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D121" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>agricultural</t>
+          <t>complex networks</t>
         </is>
       </c>
       <c r="B122" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C122" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D122" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>nacional</t>
+          <t>feature</t>
         </is>
       </c>
       <c r="B123" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C123" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D123" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>facial</t>
+          <t>event</t>
         </is>
       </c>
       <c r="B124" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C124" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D124" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>sul</t>
+          <t>fine-tuning</t>
         </is>
       </c>
       <c r="B125" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C125" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D125" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>fake news</t>
+          <t>bayesian</t>
         </is>
       </c>
       <c r="B126" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C126" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D126" t="n">
         <v>5</v>
@@ -2441,398 +2441,398 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>fake</t>
+          <t>universal</t>
         </is>
       </c>
       <c r="B127" t="n">
-        <v>5</v>
+        <v>32</v>
       </c>
       <c r="C127" t="n">
         <v>3</v>
       </c>
       <c r="D127" t="n">
-        <v>5</v>
+        <v>23</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>events</t>
+          <t>dependencies</t>
         </is>
       </c>
       <c r="B128" t="n">
-        <v>5</v>
+        <v>31</v>
       </c>
       <c r="C128" t="n">
         <v>3</v>
       </c>
       <c r="D128" t="n">
-        <v>8</v>
+        <v>24</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>computacional</t>
+          <t>universal dependencies</t>
         </is>
       </c>
       <c r="B129" t="n">
-        <v>5</v>
+        <v>29</v>
       </c>
       <c r="C129" t="n">
         <v>3</v>
       </c>
       <c r="D129" t="n">
-        <v>6</v>
+        <v>23</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>multi-objective</t>
+          <t>português</t>
         </is>
       </c>
       <c r="B130" t="n">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="C130" t="n">
         <v>3</v>
       </c>
       <c r="D130" t="n">
-        <v>3</v>
+        <v>27</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>agricultura digital</t>
+          <t>brasileiro</t>
         </is>
       </c>
       <c r="B131" t="n">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="C131" t="n">
         <v>3</v>
       </c>
       <c r="D131" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>extrusion</t>
+          <t>september</t>
         </is>
       </c>
       <c r="B132" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="C132" t="n">
         <v>3</v>
       </c>
       <c r="D132" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>algorithms</t>
+          <t>brasil</t>
         </is>
       </c>
       <c r="B133" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="C133" t="n">
         <v>3</v>
       </c>
       <c r="D133" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>reconhecimento</t>
+          <t>tweets</t>
         </is>
       </c>
       <c r="B134" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C134" t="n">
         <v>3</v>
       </c>
       <c r="D134" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>agricultura</t>
+          <t>dados</t>
         </is>
       </c>
       <c r="B135" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C135" t="n">
         <v>3</v>
       </c>
       <c r="D135" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>early</t>
+          <t>texts</t>
         </is>
       </c>
       <c r="B136" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C136" t="n">
         <v>3</v>
       </c>
       <c r="D136" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>evolutionary</t>
+          <t>estudo</t>
         </is>
       </c>
       <c r="B137" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C137" t="n">
         <v>3</v>
       </c>
       <c r="D137" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>languages</t>
+          <t>opinion</t>
         </is>
       </c>
       <c r="B138" t="n">
-        <v>19</v>
+        <v>7</v>
       </c>
       <c r="C138" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D138" t="n">
-        <v>23</v>
+        <v>4</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>indigenous</t>
+          <t>portugues</t>
         </is>
       </c>
       <c r="B139" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="C139" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D139" t="n">
-        <v>19</v>
+        <v>6</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>indigenous languages</t>
+          <t>mercado</t>
         </is>
       </c>
       <c r="B140" t="n">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="C140" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D140" t="n">
-        <v>19</v>
+        <v>6</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>prediction</t>
+          <t>lexical</t>
         </is>
       </c>
       <c r="B141" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="C141" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D141" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>parsing</t>
         </is>
       </c>
       <c r="B142" t="n">
+        <v>6</v>
+      </c>
+      <c r="C142" t="n">
+        <v>3</v>
+      </c>
+      <c r="D142" t="n">
         <v>10</v>
-      </c>
-      <c r="C142" t="n">
-        <v>4</v>
-      </c>
-      <c r="D142" t="n">
-        <v>7</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>social</t>
+          <t>mercado financeiro</t>
         </is>
       </c>
       <c r="B143" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="C143" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D143" t="n">
-        <v>13</v>
+        <v>6</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>research</t>
+          <t>financeiro</t>
         </is>
       </c>
       <c r="B144" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="C144" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D144" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>impact</t>
+          <t>construções</t>
         </is>
       </c>
       <c r="B145" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C145" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D145" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>ethical</t>
+          <t>português brasileiro</t>
         </is>
       </c>
       <c r="B146" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C146" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D146" t="n">
-        <v>14</v>
+        <v>4</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>training</t>
+          <t>linguagem</t>
         </is>
       </c>
       <c r="B147" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C147" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D147" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>brazilian indigenous</t>
+          <t>análise</t>
         </is>
       </c>
       <c r="B148" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C148" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D148" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>media</t>
+          <t>caso</t>
         </is>
       </c>
       <c r="B149" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C149" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D149" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>identification</t>
+          <t>annotation</t>
         </is>
       </c>
       <c r="B150" t="n">
         <v>5</v>
       </c>
       <c r="C150" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D150" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>human</t>
+          <t>informação</t>
         </is>
       </c>
       <c r="B151" t="n">
         <v>5</v>
       </c>
       <c r="C151" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D151" t="n">
         <v>4</v>
@@ -2841,46 +2841,46 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>smart</t>
+          <t>segundo</t>
         </is>
       </c>
       <c r="B152" t="n">
         <v>5</v>
       </c>
       <c r="C152" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D152" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>evaluating</t>
+          <t>portuguese texts</t>
         </is>
       </c>
       <c r="B153" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C153" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D153" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>social media</t>
+          <t>relações</t>
         </is>
       </c>
       <c r="B154" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C154" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D154" t="n">
         <v>5</v>
@@ -2889,353 +2889,353 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>community</t>
+          <t>processamento</t>
         </is>
       </c>
       <c r="B155" t="n">
         <v>4</v>
       </c>
       <c r="C155" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D155" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>smart toy</t>
+          <t>annotated</t>
         </is>
       </c>
       <c r="B156" t="n">
         <v>4</v>
       </c>
       <c r="C156" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D156" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>endangered</t>
+          <t>abralin</t>
         </is>
       </c>
       <c r="B157" t="n">
         <v>4</v>
       </c>
       <c r="C157" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D157" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>good</t>
+          <t>tweets mercado</t>
         </is>
       </c>
       <c r="B158" t="n">
         <v>4</v>
       </c>
       <c r="C158" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D158" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>quality</t>
+          <t>base</t>
         </is>
       </c>
       <c r="B159" t="n">
         <v>4</v>
       </c>
       <c r="C159" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D159" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>exploratory</t>
+          <t>learning</t>
         </is>
       </c>
       <c r="B160" t="n">
-        <v>4</v>
+        <v>37</v>
       </c>
       <c r="C160" t="n">
         <v>4</v>
       </c>
       <c r="D160" t="n">
-        <v>5</v>
+        <v>38</v>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>toy</t>
+          <t>models</t>
         </is>
       </c>
       <c r="B161" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="C161" t="n">
         <v>4</v>
       </c>
       <c r="D161" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>health</t>
+          <t>optimization</t>
         </is>
       </c>
       <c r="B162" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="C162" t="n">
         <v>4</v>
       </c>
       <c r="D162" t="n">
-        <v>4</v>
+        <v>14</v>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>articles</t>
+          <t>deep</t>
         </is>
       </c>
       <c r="B163" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="C163" t="n">
         <v>4</v>
       </c>
       <c r="D163" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>constraints</t>
+          <t>machine</t>
         </is>
       </c>
       <c r="B164" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="C164" t="n">
         <v>4</v>
       </c>
       <c r="D164" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>learning</t>
+          <t>machine learning</t>
         </is>
       </c>
       <c r="B165" t="n">
-        <v>37</v>
+        <v>10</v>
       </c>
       <c r="C165" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D165" t="n">
-        <v>38</v>
+        <v>14</v>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>detection</t>
+          <t>information</t>
         </is>
       </c>
       <c r="B166" t="n">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="C166" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D166" t="n">
-        <v>24</v>
+        <v>5</v>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>models</t>
+          <t>deep learning</t>
         </is>
       </c>
       <c r="B167" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="C167" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D167" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>deep</t>
+          <t>mining</t>
         </is>
       </c>
       <c r="B168" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="C168" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D168" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>machine</t>
+          <t>covid-</t>
         </is>
       </c>
       <c r="B169" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="C169" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D169" t="n">
-        <v>14</v>
+        <v>9</v>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>machine learning</t>
+          <t>state</t>
         </is>
       </c>
       <c r="B170" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="C170" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D170" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>information</t>
+          <t>sentiment</t>
         </is>
       </c>
       <c r="B171" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="C171" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D171" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>deep learning</t>
+          <t>textual</t>
         </is>
       </c>
       <c r="B172" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="C172" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D172" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>mining</t>
+          <t>segmentation</t>
         </is>
       </c>
       <c r="B173" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="C173" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D173" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>covid-</t>
+          <t>benchmark</t>
         </is>
       </c>
       <c r="B174" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C174" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D174" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>state</t>
+          <t>semantic</t>
         </is>
       </c>
       <c r="B175" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C175" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D175" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>semantic</t>
+          <t>forecasting</t>
         </is>
       </c>
       <c r="B176" t="n">
         <v>5</v>
       </c>
       <c r="C176" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D176" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="177">
@@ -3248,7 +3248,7 @@
         <v>5</v>
       </c>
       <c r="C177" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D177" t="n">
         <v>3</v>
@@ -3257,46 +3257,46 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>textual</t>
+          <t>state networks</t>
         </is>
       </c>
       <c r="B178" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C178" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D178" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>benchmark</t>
+          <t>citation</t>
         </is>
       </c>
       <c r="B179" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C179" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D179" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>sentiment</t>
+          <t>access</t>
         </is>
       </c>
       <c r="B180" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C180" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D180" t="n">
         <v>7</v>
@@ -3305,270 +3305,270 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>segmentation</t>
+          <t>evolutionary</t>
         </is>
       </c>
       <c r="B181" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C181" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D181" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>forecasting</t>
+          <t>echo</t>
         </is>
       </c>
       <c r="B182" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C182" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D182" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>automated</t>
+          <t>patients</t>
         </is>
       </c>
       <c r="B183" t="n">
         <v>4</v>
       </c>
       <c r="C183" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D183" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>symposium</t>
+          <t>echo state</t>
         </is>
       </c>
       <c r="B184" t="n">
         <v>4</v>
       </c>
       <c r="C184" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D184" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>echo state</t>
+          <t>multi-objective</t>
         </is>
       </c>
       <c r="B185" t="n">
         <v>4</v>
       </c>
       <c r="C185" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D185" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>access</t>
+          <t>algorithms</t>
         </is>
       </c>
       <c r="B186" t="n">
         <v>4</v>
       </c>
       <c r="C186" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D186" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>patients</t>
+          <t>symposium</t>
         </is>
       </c>
       <c r="B187" t="n">
         <v>4</v>
       </c>
       <c r="C187" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D187" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>echo</t>
+          <t>automated</t>
         </is>
       </c>
       <c r="B188" t="n">
         <v>4</v>
       </c>
       <c r="C188" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D188" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>citation</t>
+          <t>languages</t>
         </is>
       </c>
       <c r="B189" t="n">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="C189" t="n">
         <v>5</v>
       </c>
       <c r="D189" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>state networks</t>
+          <t>indigenous</t>
         </is>
       </c>
       <c r="B190" t="n">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="C190" t="n">
         <v>5</v>
       </c>
       <c r="D190" t="n">
-        <v>11</v>
+        <v>19</v>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>data</t>
+          <t>indigenous languages</t>
         </is>
       </c>
       <c r="B191" t="n">
-        <v>42</v>
+        <v>15</v>
       </c>
       <c r="C191" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D191" t="n">
-        <v>63</v>
+        <v>19</v>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>fair</t>
+          <t>prediction</t>
         </is>
       </c>
       <c r="B192" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="C192" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D192" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>natural</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B193" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C193" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D193" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>datasets</t>
+          <t>social</t>
         </is>
       </c>
       <c r="B194" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C194" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D194" t="n">
-        <v>6</v>
+        <v>13</v>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>science</t>
+          <t>research</t>
         </is>
       </c>
       <c r="B195" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C195" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D195" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>agriculture</t>
+          <t>ethical</t>
         </is>
       </c>
       <c r="B196" t="n">
         <v>7</v>
       </c>
       <c r="C196" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D196" t="n">
-        <v>5</v>
+        <v>14</v>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>computer</t>
+          <t>impact</t>
         </is>
       </c>
       <c r="B197" t="n">
         <v>7</v>
       </c>
       <c r="C197" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D197" t="n">
         <v>7</v>
@@ -3577,286 +3577,286 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>computational</t>
+          <t>brazilian indigenous</t>
         </is>
       </c>
       <c r="B198" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C198" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D198" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>applied</t>
+          <t>training</t>
         </is>
       </c>
       <c r="B199" t="n">
         <v>6</v>
       </c>
       <c r="C199" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D199" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>knowledge</t>
+          <t>media</t>
         </is>
       </c>
       <c r="B200" t="n">
         <v>6</v>
       </c>
       <c r="C200" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D200" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>natural language</t>
+          <t>social media</t>
         </is>
       </c>
       <c r="B201" t="n">
         <v>5</v>
       </c>
       <c r="C201" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D201" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>data augmentation</t>
+          <t>human</t>
         </is>
       </c>
       <c r="B202" t="n">
         <v>5</v>
       </c>
       <c r="C202" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D202" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>set</t>
+          <t>evaluating</t>
         </is>
       </c>
       <c r="B203" t="n">
         <v>5</v>
       </c>
       <c r="C203" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D203" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>augmentation</t>
+          <t>identification</t>
         </is>
       </c>
       <c r="B204" t="n">
         <v>5</v>
       </c>
       <c r="C204" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D204" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>formal</t>
+          <t>smart</t>
         </is>
       </c>
       <c r="B205" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C205" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D205" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>building</t>
+          <t>constraints</t>
         </is>
       </c>
       <c r="B206" t="n">
         <v>4</v>
       </c>
       <c r="C206" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D206" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>low-resource</t>
+          <t>good</t>
         </is>
       </c>
       <c r="B207" t="n">
         <v>4</v>
       </c>
       <c r="C207" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D207" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>blue amazon</t>
+          <t>exploratory</t>
         </is>
       </c>
       <c r="B208" t="n">
         <v>4</v>
       </c>
       <c r="C208" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D208" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>philosophy</t>
+          <t>articles</t>
         </is>
       </c>
       <c r="B209" t="n">
         <v>4</v>
       </c>
       <c r="C209" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D209" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>probabilistic</t>
+          <t>smart toy</t>
         </is>
       </c>
       <c r="B210" t="n">
         <v>4</v>
       </c>
       <c r="C210" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D210" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>blue</t>
+          <t>quality</t>
         </is>
       </c>
       <c r="B211" t="n">
         <v>4</v>
       </c>
       <c r="C211" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D211" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>build</t>
+          <t>toy</t>
         </is>
       </c>
       <c r="B212" t="n">
         <v>4</v>
       </c>
       <c r="C212" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D212" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>diagnosis</t>
+          <t>community</t>
         </is>
       </c>
       <c r="B213" t="n">
         <v>4</v>
       </c>
       <c r="C213" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D213" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>data intelligence</t>
+          <t>health</t>
         </is>
       </c>
       <c r="B214" t="n">
         <v>4</v>
       </c>
       <c r="C214" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D214" t="n">
-        <v>14</v>
+        <v>4</v>
       </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>amazon</t>
+          <t>endangered</t>
         </is>
       </c>
       <c r="B215" t="n">
         <v>4</v>
       </c>
       <c r="C215" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D215" t="n">
         <v>8</v>
@@ -3872,7 +3872,7 @@
         <v>12</v>
       </c>
       <c r="C216" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D216" t="n">
         <v>18</v>
@@ -3888,7 +3888,7 @@
         <v>10</v>
       </c>
       <c r="C217" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D217" t="n">
         <v>16</v>
@@ -3904,7 +3904,7 @@
         <v>9</v>
       </c>
       <c r="C218" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D218" t="n">
         <v>18</v>
@@ -3920,7 +3920,7 @@
         <v>9</v>
       </c>
       <c r="C219" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D219" t="n">
         <v>14</v>
@@ -3936,7 +3936,7 @@
         <v>8</v>
       </c>
       <c r="C220" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D220" t="n">
         <v>15</v>
@@ -3952,7 +3952,7 @@
         <v>7</v>
       </c>
       <c r="C221" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D221" t="n">
         <v>11</v>
@@ -3968,7 +3968,7 @@
         <v>6</v>
       </c>
       <c r="C222" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D222" t="n">
         <v>12</v>
@@ -3984,7 +3984,7 @@
         <v>5</v>
       </c>
       <c r="C223" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D223" t="n">
         <v>7</v>
@@ -3993,94 +3993,94 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>chatgpt</t>
+          <t>time series</t>
         </is>
       </c>
       <c r="B224" t="n">
         <v>4</v>
       </c>
       <c r="C224" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D224" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>series</t>
+          <t>oceanic</t>
         </is>
       </c>
       <c r="B225" t="n">
         <v>4</v>
       </c>
       <c r="C225" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D225" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>oceanic variables</t>
+          <t>assessing</t>
         </is>
       </c>
       <c r="B226" t="n">
         <v>4</v>
       </c>
       <c r="C226" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D226" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>oceans</t>
+          <t>chatgpt</t>
         </is>
       </c>
       <c r="B227" t="n">
         <v>4</v>
       </c>
       <c r="C227" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D227" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>assessing</t>
+          <t>series</t>
         </is>
       </c>
       <c r="B228" t="n">
         <v>4</v>
       </c>
       <c r="C228" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D228" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>oceanic</t>
+          <t>oceanic variables</t>
         </is>
       </c>
       <c r="B229" t="n">
         <v>4</v>
       </c>
       <c r="C229" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D229" t="n">
         <v>11</v>
@@ -4089,30 +4089,30 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>time series</t>
+          <t>oceans</t>
         </is>
       </c>
       <c r="B230" t="n">
         <v>4</v>
       </c>
       <c r="C230" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D230" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>multiple</t>
+          <t>porttinari</t>
         </is>
       </c>
       <c r="B231" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C231" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D231" t="n">
         <v>1</v>
@@ -4121,14 +4121,14 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>within</t>
+          <t>treebank</t>
         </is>
       </c>
       <c r="B232" t="n">
         <v>4</v>
       </c>
       <c r="C232" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D232" t="n">
         <v>1</v>
@@ -4137,14 +4137,14 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>treebank</t>
+          <t>multiple</t>
         </is>
       </c>
       <c r="B233" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C233" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D233" t="n">
         <v>1</v>
@@ -4153,14 +4153,14 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>porttinari</t>
+          <t>within</t>
         </is>
       </c>
       <c r="B234" t="n">
         <v>4</v>
       </c>
       <c r="C234" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D234" t="n">
         <v>1</v>

</xml_diff>

<commit_message>
Espalha os nós da rede de co-ocorrência (menos amontoados)
- coword_analysis.py: aumenta a repulsão do layout (k maior) e usa escala por
  raiz quadrada no tamanho dos nós, evitando bolas enormes e o amontoamento no
  centro. Mesmo ajuste nos painéis temporais.
- Regenera Figuras 10 e 11.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Fvrdaa5i99DsPUToDczGGv
</commit_message>
<xml_diff>
--- a/output/coword/coword_nos_comunidades.xlsx
+++ b/output/coword/coword_nos_comunidades.xlsx
@@ -537,7 +537,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ocean</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -547,13 +547,13 @@
         <v>0</v>
       </c>
       <c r="D8" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>dynamic</t>
+          <t>ocean</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -563,7 +563,7 @@
         <v>0</v>
       </c>
       <c r="D9" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="10">
@@ -617,7 +617,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>engineering</t>
+          <t>state</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -627,7 +627,7 @@
         <v>0</v>
       </c>
       <c r="D13" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
     </row>
     <row r="14">
@@ -665,7 +665,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>state</t>
+          <t>engineering</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -675,7 +675,7 @@
         <v>0</v>
       </c>
       <c r="D16" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="17">
@@ -697,7 +697,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>assessment</t>
+          <t>textual</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -707,13 +707,13 @@
         <v>0</v>
       </c>
       <c r="D18" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>arctic</t>
+          <t>offshore</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -729,7 +729,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>resilience</t>
+          <t>arctic</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -739,13 +739,13 @@
         <v>0</v>
       </c>
       <c r="D20" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>physics-informed neural</t>
+          <t>resilience</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -761,7 +761,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>textual</t>
+          <t>selection</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -771,7 +771,7 @@
         <v>0</v>
       </c>
       <c r="D22" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="23">
@@ -793,7 +793,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>offshore</t>
+          <t>estimation</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -803,13 +803,13 @@
         <v>0</v>
       </c>
       <c r="D24" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>propagation</t>
+          <t>physics-informed neural</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -819,13 +819,13 @@
         <v>0</v>
       </c>
       <c r="D25" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>selection</t>
+          <t>assessment</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -835,13 +835,13 @@
         <v>0</v>
       </c>
       <c r="D26" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>estimation</t>
+          <t>propagation</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -851,13 +851,13 @@
         <v>0</v>
       </c>
       <c r="D27" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>ocean offshore</t>
+          <t>echo state</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -867,13 +867,13 @@
         <v>0</v>
       </c>
       <c r="D28" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>fine-tuning</t>
+          <t>insurance</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -883,13 +883,13 @@
         <v>0</v>
       </c>
       <c r="D29" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>index</t>
+          <t>operator</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -899,13 +899,13 @@
         <v>0</v>
       </c>
       <c r="D30" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>echo</t>
+          <t>event</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -915,13 +915,13 @@
         <v>0</v>
       </c>
       <c r="D31" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>insurance</t>
+          <t>synchronization</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -931,13 +931,13 @@
         <v>0</v>
       </c>
       <c r="D32" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>event</t>
+          <t>state networks</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -947,13 +947,13 @@
         <v>0</v>
       </c>
       <c r="D33" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>state networks</t>
+          <t>bayesian</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -963,13 +963,13 @@
         <v>0</v>
       </c>
       <c r="D34" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>semi-supervised</t>
+          <t>forecasting</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -979,13 +979,13 @@
         <v>0</v>
       </c>
       <c r="D35" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>forecasting</t>
+          <t>feature</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -995,13 +995,13 @@
         <v>0</v>
       </c>
       <c r="D36" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>echo state</t>
+          <t>semi-supervised</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1011,7 +1011,7 @@
         <v>0</v>
       </c>
       <c r="D37" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="38">
@@ -1033,7 +1033,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>synchronization</t>
+          <t>echo</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1043,13 +1043,13 @@
         <v>0</v>
       </c>
       <c r="D39" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>feature</t>
+          <t>ocean offshore</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1059,13 +1059,13 @@
         <v>0</v>
       </c>
       <c r="D40" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>bayesian</t>
+          <t>fine-tuning</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1075,13 +1075,13 @@
         <v>0</v>
       </c>
       <c r="D41" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>neural operator</t>
+          <t>index</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -1091,13 +1091,13 @@
         <v>0</v>
       </c>
       <c r="D42" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>operator</t>
+          <t>neural operator</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -1193,7 +1193,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>optimization</t>
+          <t>inteligência</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -1203,7 +1203,7 @@
         <v>1</v>
       </c>
       <c r="D49" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
     </row>
     <row r="50">
@@ -1225,7 +1225,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>inteligência</t>
+          <t>optimization</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -1235,13 +1235,13 @@
         <v>1</v>
       </c>
       <c r="D51" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>processing</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -1251,7 +1251,7 @@
         <v>1</v>
       </c>
       <c r="D52" t="n">
-        <v>21</v>
+        <v>6</v>
       </c>
     </row>
     <row r="53">
@@ -1273,7 +1273,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>datasets</t>
+          <t>fair</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -1283,77 +1283,77 @@
         <v>1</v>
       </c>
       <c r="D54" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>multimodal</t>
+          <t>opinion</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C55" t="n">
         <v>1</v>
       </c>
       <c r="D55" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>agricultural</t>
+          <t>datasets</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C56" t="n">
         <v>1</v>
       </c>
       <c r="D56" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>fake</t>
+          <t>multimodal</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C57" t="n">
         <v>1</v>
       </c>
       <c r="D57" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>events</t>
+          <t>agricultural</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C58" t="n">
         <v>1</v>
       </c>
       <c r="D58" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>data augmentation</t>
+          <t>events</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -1363,13 +1363,13 @@
         <v>1</v>
       </c>
       <c r="D59" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>mining</t>
+          <t>set</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -1379,7 +1379,7 @@
         <v>1</v>
       </c>
       <c r="D60" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="61">
@@ -1401,7 +1401,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>augmentation</t>
+          <t>applied</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -1417,7 +1417,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>applied</t>
+          <t>mining</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -1427,77 +1427,77 @@
         <v>1</v>
       </c>
       <c r="D63" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>extrusion</t>
+          <t>agriculture</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C64" t="n">
         <v>1</v>
       </c>
       <c r="D64" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>algorithms</t>
+          <t>data augmentation</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C65" t="n">
         <v>1</v>
       </c>
       <c r="D65" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>computacional</t>
+          <t>fake</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C66" t="n">
         <v>1</v>
       </c>
       <c r="D66" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>multi-objective</t>
+          <t>augmentation</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C67" t="n">
         <v>1</v>
       </c>
       <c r="D67" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>data intelligence</t>
+          <t>extrusion</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -1507,13 +1507,13 @@
         <v>1</v>
       </c>
       <c r="D68" t="n">
-        <v>14</v>
+        <v>6</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>early</t>
+          <t>facial</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -1523,13 +1523,13 @@
         <v>1</v>
       </c>
       <c r="D69" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>amazon</t>
+          <t>build</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -1539,13 +1539,13 @@
         <v>1</v>
       </c>
       <c r="D70" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>build</t>
+          <t>computacional</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -1555,13 +1555,13 @@
         <v>1</v>
       </c>
       <c r="D71" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>facial</t>
+          <t>building</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -1577,7 +1577,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>blue</t>
+          <t>knowledge</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -1593,7 +1593,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>low-resource</t>
+          <t>blue</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -1603,13 +1603,13 @@
         <v>1</v>
       </c>
       <c r="D74" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>blue amazon</t>
+          <t>algorithms</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -1619,13 +1619,13 @@
         <v>1</v>
       </c>
       <c r="D75" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>knowledge</t>
+          <t>low-resource</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -1635,461 +1635,461 @@
         <v>1</v>
       </c>
       <c r="D76" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>brazilian</t>
+          <t>amazon</t>
         </is>
       </c>
       <c r="B77" t="n">
-        <v>53</v>
+        <v>4</v>
       </c>
       <c r="C77" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D77" t="n">
-        <v>66</v>
+        <v>8</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>portuguese</t>
+          <t>data intelligence</t>
         </is>
       </c>
       <c r="B78" t="n">
-        <v>50</v>
+        <v>4</v>
       </c>
       <c r="C78" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D78" t="n">
-        <v>50</v>
+        <v>14</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>speech</t>
+          <t>blue amazon</t>
         </is>
       </c>
       <c r="B79" t="n">
-        <v>22</v>
+        <v>4</v>
       </c>
       <c r="C79" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D79" t="n">
-        <v>35</v>
+        <v>8</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>language</t>
+          <t>early</t>
         </is>
       </c>
       <c r="B80" t="n">
-        <v>21</v>
+        <v>4</v>
       </c>
       <c r="C80" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D80" t="n">
-        <v>26</v>
+        <v>8</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>brazilian portuguese</t>
+          <t>multi-objective</t>
         </is>
       </c>
       <c r="B81" t="n">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="C81" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D81" t="n">
-        <v>22</v>
+        <v>3</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>corpus</t>
+          <t>brazilian</t>
         </is>
       </c>
       <c r="B82" t="n">
-        <v>18</v>
+        <v>53</v>
       </c>
       <c r="C82" t="n">
         <v>2</v>
       </c>
       <c r="D82" t="n">
-        <v>28</v>
+        <v>66</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>evaluation</t>
+          <t>portuguese</t>
         </is>
       </c>
       <c r="B83" t="n">
-        <v>15</v>
+        <v>50</v>
       </c>
       <c r="C83" t="n">
         <v>2</v>
       </c>
       <c r="D83" t="n">
-        <v>25</v>
+        <v>50</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>recognition</t>
+          <t>speech</t>
         </is>
       </c>
       <c r="B84" t="n">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="C84" t="n">
         <v>2</v>
       </c>
       <c r="D84" t="n">
-        <v>23</v>
+        <v>35</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>intelligent</t>
+          <t>language</t>
         </is>
       </c>
       <c r="B85" t="n">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="C85" t="n">
         <v>2</v>
       </c>
       <c r="D85" t="n">
-        <v>11</v>
+        <v>26</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>resources</t>
+          <t>brazilian portuguese</t>
         </is>
       </c>
       <c r="B86" t="n">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="C86" t="n">
         <v>2</v>
       </c>
       <c r="D86" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>automatic</t>
+          <t>corpus</t>
         </is>
       </c>
       <c r="B87" t="n">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="C87" t="n">
         <v>2</v>
       </c>
       <c r="D87" t="n">
-        <v>8</v>
+        <v>28</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>bracis</t>
+          <t>evaluation</t>
         </is>
       </c>
       <c r="B88" t="n">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="C88" t="n">
         <v>2</v>
       </c>
       <c r="D88" t="n">
-        <v>4</v>
+        <v>25</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>speech recognition</t>
+          <t>recognition</t>
         </is>
       </c>
       <c r="B89" t="n">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="C89" t="n">
         <v>2</v>
       </c>
       <c r="D89" t="n">
-        <v>13</v>
+        <v>23</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>public</t>
+          <t>intelligent</t>
         </is>
       </c>
       <c r="B90" t="n">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="C90" t="n">
         <v>2</v>
       </c>
       <c r="D90" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>asr</t>
+          <t>automatic</t>
         </is>
       </c>
       <c r="B91" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="C91" t="n">
         <v>2</v>
       </c>
       <c r="D91" t="n">
-        <v>19</v>
+        <v>8</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>spontaneous</t>
+          <t>processing</t>
         </is>
       </c>
       <c r="B92" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="C92" t="n">
         <v>2</v>
       </c>
       <c r="D92" t="n">
-        <v>13</v>
+        <v>21</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>design</t>
+          <t>resources</t>
         </is>
       </c>
       <c r="B93" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="C93" t="n">
         <v>2</v>
       </c>
       <c r="D93" t="n">
-        <v>13</v>
+        <v>24</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>cham</t>
+          <t>natural</t>
         </is>
       </c>
       <c r="B94" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C94" t="n">
         <v>2</v>
       </c>
       <c r="D94" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>extraction</t>
+          <t>bracis</t>
         </is>
       </c>
       <c r="B95" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C95" t="n">
         <v>2</v>
       </c>
       <c r="D95" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>portuguese language</t>
+          <t>asr</t>
         </is>
       </c>
       <c r="B96" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C96" t="n">
         <v>2</v>
       </c>
       <c r="D96" t="n">
-        <v>8</v>
+        <v>19</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>coraa</t>
+          <t>spontaneous</t>
         </is>
       </c>
       <c r="B97" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C97" t="n">
         <v>2</v>
       </c>
       <c r="D97" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>emotion</t>
+          <t>public</t>
         </is>
       </c>
       <c r="B98" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C98" t="n">
         <v>2</v>
       </c>
       <c r="D98" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>features</t>
+          <t>speech recognition</t>
         </is>
       </c>
       <c r="B99" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C99" t="n">
         <v>2</v>
       </c>
       <c r="D99" t="n">
-        <v>6</v>
+        <v>13</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>online</t>
+          <t>cham</t>
         </is>
       </c>
       <c r="B100" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C100" t="n">
         <v>2</v>
       </c>
       <c r="D100" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>spoken</t>
+          <t>design</t>
         </is>
       </c>
       <c r="B101" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C101" t="n">
         <v>2</v>
       </c>
       <c r="D101" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>emotion recognition</t>
+          <t>extraction</t>
         </is>
       </c>
       <c r="B102" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C102" t="n">
         <v>2</v>
       </c>
       <c r="D102" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>manually</t>
+          <t>portuguese language</t>
         </is>
       </c>
       <c r="B103" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C103" t="n">
         <v>2</v>
       </c>
       <c r="D103" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>corpora</t>
+          <t>natural language</t>
         </is>
       </c>
       <c r="B104" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C104" t="n">
         <v>2</v>
       </c>
       <c r="D104" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>latin</t>
+          <t>formal</t>
         </is>
       </c>
       <c r="B105" t="n">
@@ -2099,13 +2099,13 @@
         <v>2</v>
       </c>
       <c r="D105" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>development</t>
+          <t>manually</t>
         </is>
       </c>
       <c r="B106" t="n">
@@ -2115,321 +2115,321 @@
         <v>2</v>
       </c>
       <c r="D106" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>languages</t>
+          <t>emotion</t>
         </is>
       </c>
       <c r="B107" t="n">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="C107" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D107" t="n">
-        <v>21</v>
+        <v>5</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>indigenous</t>
+          <t>corpora</t>
         </is>
       </c>
       <c r="B108" t="n">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="C108" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D108" t="n">
-        <v>18</v>
+        <v>12</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>indigenous languages</t>
+          <t>coraa</t>
         </is>
       </c>
       <c r="B109" t="n">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="C109" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D109" t="n">
-        <v>18</v>
+        <v>12</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>prediction</t>
+          <t>probabilistic</t>
         </is>
       </c>
       <c r="B110" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="C110" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D110" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>social</t>
+          <t>online</t>
         </is>
       </c>
       <c r="B111" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="C111" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D111" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>ethical</t>
+          <t>development</t>
         </is>
       </c>
       <c r="B112" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C112" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D112" t="n">
-        <v>14</v>
+        <v>9</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>impact</t>
+          <t>emotion recognition</t>
         </is>
       </c>
       <c r="B113" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C113" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D113" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>brazilian indigenous</t>
+          <t>latin</t>
         </is>
       </c>
       <c r="B114" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C114" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D114" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>training</t>
+          <t>features</t>
         </is>
       </c>
       <c r="B115" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C115" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D115" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>media</t>
+          <t>science</t>
         </is>
       </c>
       <c r="B116" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C116" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D116" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>smart</t>
+          <t>computer</t>
         </is>
       </c>
       <c r="B117" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C117" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D117" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>evaluating</t>
+          <t>spoken</t>
         </is>
       </c>
       <c r="B118" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C118" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D118" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>identification</t>
+          <t>universal</t>
         </is>
       </c>
       <c r="B119" t="n">
-        <v>5</v>
+        <v>32</v>
       </c>
       <c r="C119" t="n">
         <v>3</v>
       </c>
       <c r="D119" t="n">
-        <v>6</v>
+        <v>23</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>social media</t>
+          <t>dependencies</t>
         </is>
       </c>
       <c r="B120" t="n">
-        <v>5</v>
+        <v>31</v>
       </c>
       <c r="C120" t="n">
         <v>3</v>
       </c>
       <c r="D120" t="n">
-        <v>4</v>
+        <v>24</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>human</t>
+          <t>universal dependencies</t>
         </is>
       </c>
       <c r="B121" t="n">
-        <v>4</v>
+        <v>29</v>
       </c>
       <c r="C121" t="n">
         <v>3</v>
       </c>
       <c r="D121" t="n">
-        <v>4</v>
+        <v>23</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>exploratory</t>
+          <t>português</t>
         </is>
       </c>
       <c r="B122" t="n">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="C122" t="n">
         <v>3</v>
       </c>
       <c r="D122" t="n">
-        <v>5</v>
+        <v>27</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>smart toy</t>
+          <t>brasileiro</t>
         </is>
       </c>
       <c r="B123" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="C123" t="n">
         <v>3</v>
       </c>
       <c r="D123" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>research</t>
+          <t>dados</t>
         </is>
       </c>
       <c r="B124" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="C124" t="n">
         <v>3</v>
       </c>
       <c r="D124" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>toy</t>
+          <t>september</t>
         </is>
       </c>
       <c r="B125" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C125" t="n">
         <v>3</v>
       </c>
       <c r="D125" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>constraints</t>
+          <t>tweets</t>
         </is>
       </c>
       <c r="B126" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C126" t="n">
         <v>3</v>
@@ -2441,238 +2441,238 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>community</t>
+          <t>texts</t>
         </is>
       </c>
       <c r="B127" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C127" t="n">
         <v>3</v>
       </c>
       <c r="D127" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>articles</t>
+          <t>brasil</t>
         </is>
       </c>
       <c r="B128" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C128" t="n">
         <v>3</v>
       </c>
       <c r="D128" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>good</t>
+          <t>portugues</t>
         </is>
       </c>
       <c r="B129" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C129" t="n">
         <v>3</v>
       </c>
       <c r="D129" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>endangered</t>
+          <t>estudo</t>
         </is>
       </c>
       <c r="B130" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C130" t="n">
         <v>3</v>
       </c>
       <c r="D130" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>universal</t>
+          <t>lexical</t>
         </is>
       </c>
       <c r="B131" t="n">
-        <v>32</v>
+        <v>6</v>
       </c>
       <c r="C131" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D131" t="n">
-        <v>23</v>
+        <v>4</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>dependencies</t>
+          <t>mercado</t>
         </is>
       </c>
       <c r="B132" t="n">
-        <v>31</v>
+        <v>6</v>
       </c>
       <c r="C132" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D132" t="n">
-        <v>24</v>
+        <v>6</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>universal dependencies</t>
+          <t>parsing</t>
         </is>
       </c>
       <c r="B133" t="n">
-        <v>29</v>
+        <v>6</v>
       </c>
       <c r="C133" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D133" t="n">
-        <v>23</v>
+        <v>10</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>português</t>
+          <t>mercado financeiro</t>
         </is>
       </c>
       <c r="B134" t="n">
-        <v>23</v>
+        <v>6</v>
       </c>
       <c r="C134" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D134" t="n">
-        <v>27</v>
+        <v>6</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>brasileiro</t>
+          <t>financeiro</t>
         </is>
       </c>
       <c r="B135" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="C135" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D135" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>september</t>
+          <t>construções</t>
         </is>
       </c>
       <c r="B136" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C136" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D136" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>estudo</t>
+          <t>annotation</t>
         </is>
       </c>
       <c r="B137" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C137" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D137" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>texts</t>
+          <t>segundo</t>
         </is>
       </c>
       <c r="B138" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C138" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D138" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>portugues</t>
+          <t>análise</t>
         </is>
       </c>
       <c r="B139" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C139" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D139" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>brasil</t>
+          <t>linguagem</t>
         </is>
       </c>
       <c r="B140" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C140" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D140" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>construções</t>
+          <t>caso</t>
         </is>
       </c>
       <c r="B141" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C141" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D141" t="n">
         <v>8</v>
@@ -2681,14 +2681,14 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>lexical</t>
+          <t>português brasileiro</t>
         </is>
       </c>
       <c r="B142" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C142" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D142" t="n">
         <v>4</v>
@@ -2697,222 +2697,222 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>parsing</t>
+          <t>abralin</t>
         </is>
       </c>
       <c r="B143" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C143" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D143" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>annotation</t>
+          <t>portuguese texts</t>
         </is>
       </c>
       <c r="B144" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C144" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D144" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>segundo</t>
+          <t>processamento</t>
         </is>
       </c>
       <c r="B145" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C145" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D145" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>análise</t>
+          <t>tweets mercado</t>
         </is>
       </c>
       <c r="B146" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C146" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D146" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>linguagem</t>
+          <t>relações</t>
         </is>
       </c>
       <c r="B147" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C147" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D147" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>português brasileiro</t>
+          <t>annotated</t>
         </is>
       </c>
       <c r="B148" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C148" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D148" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>portuguese texts</t>
+          <t>informação</t>
         </is>
       </c>
       <c r="B149" t="n">
         <v>4</v>
       </c>
       <c r="C149" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D149" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>informação</t>
+          <t>languages</t>
         </is>
       </c>
       <c r="B150" t="n">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="C150" t="n">
         <v>4</v>
       </c>
       <c r="D150" t="n">
-        <v>4</v>
+        <v>21</v>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>annotated</t>
+          <t>indigenous</t>
         </is>
       </c>
       <c r="B151" t="n">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="C151" t="n">
         <v>4</v>
       </c>
       <c r="D151" t="n">
-        <v>9</v>
+        <v>18</v>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>abralin</t>
+          <t>indigenous languages</t>
         </is>
       </c>
       <c r="B152" t="n">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="C152" t="n">
         <v>4</v>
       </c>
       <c r="D152" t="n">
-        <v>5</v>
+        <v>18</v>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>relações</t>
+          <t>prediction</t>
         </is>
       </c>
       <c r="B153" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="C153" t="n">
         <v>4</v>
       </c>
       <c r="D153" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>processamento</t>
+          <t>social</t>
         </is>
       </c>
       <c r="B154" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="C154" t="n">
         <v>4</v>
       </c>
       <c r="D154" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>modeling</t>
+          <t>impact</t>
         </is>
       </c>
       <c r="B155" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="C155" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D155" t="n">
-        <v>18</v>
+        <v>7</v>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>dataset</t>
+          <t>ethical</t>
         </is>
       </c>
       <c r="B156" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="C156" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D156" t="n">
         <v>14</v>
@@ -2921,318 +2921,318 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>model</t>
+          <t>media</t>
         </is>
       </c>
       <c r="B157" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="C157" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D157" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>climate</t>
+          <t>training</t>
         </is>
       </c>
       <c r="B158" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="C158" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D158" t="n">
-        <v>16</v>
+        <v>5</v>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>change</t>
+          <t>brazilian indigenous</t>
         </is>
       </c>
       <c r="B159" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C159" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D159" t="n">
-        <v>18</v>
+        <v>9</v>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>climate change</t>
+          <t>smart</t>
         </is>
       </c>
       <c r="B160" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C160" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D160" t="n">
-        <v>15</v>
+        <v>5</v>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>variables</t>
+          <t>evaluating</t>
         </is>
       </c>
       <c r="B161" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C161" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D161" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>time</t>
+          <t>identification</t>
         </is>
       </c>
       <c r="B162" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C162" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D162" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>tasks</t>
+          <t>social media</t>
         </is>
       </c>
       <c r="B163" t="n">
         <v>5</v>
       </c>
       <c r="C163" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D163" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>chatgpt</t>
+          <t>human</t>
         </is>
       </c>
       <c r="B164" t="n">
         <v>4</v>
       </c>
       <c r="C164" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D164" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>time series</t>
+          <t>toy</t>
         </is>
       </c>
       <c r="B165" t="n">
         <v>4</v>
       </c>
       <c r="C165" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D165" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>oceanic</t>
+          <t>constraints</t>
         </is>
       </c>
       <c r="B166" t="n">
         <v>4</v>
       </c>
       <c r="C166" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D166" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>assessing</t>
+          <t>research</t>
         </is>
       </c>
       <c r="B167" t="n">
         <v>4</v>
       </c>
       <c r="C167" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D167" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>series</t>
+          <t>community</t>
         </is>
       </c>
       <c r="B168" t="n">
         <v>4</v>
       </c>
       <c r="C168" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D168" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>oceanic variables</t>
+          <t>endangered</t>
         </is>
       </c>
       <c r="B169" t="n">
         <v>4</v>
       </c>
       <c r="C169" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D169" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>oceans</t>
+          <t>exploratory</t>
         </is>
       </c>
       <c r="B170" t="n">
         <v>4</v>
       </c>
       <c r="C170" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D170" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>learning</t>
+          <t>good</t>
         </is>
       </c>
       <c r="B171" t="n">
-        <v>33</v>
+        <v>4</v>
       </c>
       <c r="C171" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D171" t="n">
-        <v>24</v>
+        <v>11</v>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>models</t>
+          <t>smart toy</t>
         </is>
       </c>
       <c r="B172" t="n">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="C172" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D172" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>deep</t>
+          <t>articles</t>
         </is>
       </c>
       <c r="B173" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="C173" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D173" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>machine</t>
+          <t>modeling</t>
         </is>
       </c>
       <c r="B174" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C174" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D174" t="n">
-        <v>8</v>
+        <v>18</v>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>machine learning</t>
+          <t>dataset</t>
         </is>
       </c>
       <c r="B175" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C175" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D175" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>deep learning</t>
+          <t>model</t>
         </is>
       </c>
       <c r="B176" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C176" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D176" t="n">
         <v>6</v>
@@ -3241,94 +3241,94 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>covid-</t>
+          <t>climate</t>
         </is>
       </c>
       <c r="B177" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C177" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D177" t="n">
-        <v>5</v>
+        <v>16</v>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>segmentation</t>
+          <t>change</t>
         </is>
       </c>
       <c r="B178" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C178" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D178" t="n">
-        <v>5</v>
+        <v>18</v>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>representation</t>
+          <t>climate change</t>
         </is>
       </c>
       <c r="B179" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C179" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D179" t="n">
-        <v>2</v>
+        <v>15</v>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>benchmark</t>
+          <t>time</t>
         </is>
       </c>
       <c r="B180" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C180" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D180" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>sentiment</t>
+          <t>variables</t>
         </is>
       </c>
       <c r="B181" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C181" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D181" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>automated</t>
+          <t>tasks</t>
         </is>
       </c>
       <c r="B182" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C182" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D182" t="n">
         <v>7</v>
@@ -3337,366 +3337,366 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>computational</t>
+          <t>series</t>
         </is>
       </c>
       <c r="B183" t="n">
         <v>4</v>
       </c>
       <c r="C183" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D183" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>semantic</t>
+          <t>oceanic</t>
         </is>
       </c>
       <c r="B184" t="n">
         <v>4</v>
       </c>
       <c r="C184" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D184" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>patients</t>
+          <t>chatgpt</t>
         </is>
       </c>
       <c r="B185" t="n">
         <v>4</v>
       </c>
       <c r="C185" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D185" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>dados</t>
+          <t>time series</t>
         </is>
       </c>
       <c r="B186" t="n">
+        <v>4</v>
+      </c>
+      <c r="C186" t="n">
+        <v>5</v>
+      </c>
+      <c r="D186" t="n">
         <v>8</v>
-      </c>
-      <c r="C186" t="n">
-        <v>7</v>
-      </c>
-      <c r="D186" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>tweets</t>
+          <t>oceans</t>
         </is>
       </c>
       <c r="B187" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C187" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D187" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>mercado financeiro</t>
+          <t>oceanic variables</t>
         </is>
       </c>
       <c r="B188" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C188" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D188" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>mercado</t>
+          <t>assessing</t>
         </is>
       </c>
       <c r="B189" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C189" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D189" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>financeiro</t>
+          <t>learning</t>
         </is>
       </c>
       <c r="B190" t="n">
-        <v>6</v>
+        <v>33</v>
       </c>
       <c r="C190" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D190" t="n">
-        <v>6</v>
+        <v>24</v>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>caso</t>
+          <t>models</t>
         </is>
       </c>
       <c r="B191" t="n">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="C191" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D191" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>tweets mercado</t>
+          <t>deep</t>
         </is>
       </c>
       <c r="B192" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="C192" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D192" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>natural</t>
+          <t>machine learning</t>
         </is>
       </c>
       <c r="B193" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C193" t="n">
+        <v>6</v>
+      </c>
+      <c r="D193" t="n">
         <v>8</v>
-      </c>
-      <c r="D193" t="n">
-        <v>9</v>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>natural language</t>
+          <t>machine</t>
         </is>
       </c>
       <c r="B194" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="C194" t="n">
+        <v>6</v>
+      </c>
+      <c r="D194" t="n">
         <v>8</v>
-      </c>
-      <c r="D194" t="n">
-        <v>7</v>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>probabilistic</t>
+          <t>deep learning</t>
         </is>
       </c>
       <c r="B195" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="C195" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D195" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>formal</t>
+          <t>covid-</t>
         </is>
       </c>
       <c r="B196" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C196" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D196" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>science</t>
+          <t>segmentation</t>
         </is>
       </c>
       <c r="B197" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C197" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D197" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>computer</t>
+          <t>representation</t>
         </is>
       </c>
       <c r="B198" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C198" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D198" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>benchmark</t>
         </is>
       </c>
       <c r="B199" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="C199" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D199" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>fair</t>
+          <t>sentiment</t>
         </is>
       </c>
       <c r="B200" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C200" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D200" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>opinion</t>
+          <t>computational</t>
         </is>
       </c>
       <c r="B201" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C201" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D201" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>agriculture</t>
+          <t>patients</t>
         </is>
       </c>
       <c r="B202" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C202" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D202" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>set</t>
+          <t>automated</t>
         </is>
       </c>
       <c r="B203" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C203" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D203" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>building</t>
+          <t>semantic</t>
         </is>
       </c>
       <c r="B204" t="n">
         <v>4</v>
       </c>
       <c r="C204" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D204" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>multiple</t>
+          <t>treebank</t>
         </is>
       </c>
       <c r="B205" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C205" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="D205" t="n">
         <v>1</v>
@@ -3705,14 +3705,14 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>within</t>
+          <t>porttinari</t>
         </is>
       </c>
       <c r="B206" t="n">
         <v>4</v>
       </c>
       <c r="C206" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="D206" t="n">
         <v>1</v>
@@ -3721,14 +3721,14 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>treebank</t>
+          <t>multiple</t>
         </is>
       </c>
       <c r="B207" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C207" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D207" t="n">
         <v>1</v>
@@ -3737,14 +3737,14 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>porttinari</t>
+          <t>within</t>
         </is>
       </c>
       <c r="B208" t="n">
         <v>4</v>
       </c>
       <c r="C208" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D208" t="n">
         <v>1</v>

</xml_diff>

<commit_message>
Remove títulos internos das redes de co-ocorrência (figuras 10 e 11)
Remove o título interno (set_title/suptitle) das figuras de co-word
analysis — rede global (10_rede_coword) e deslocamento temporal
(11_rede_coword_temporal) —, seguindo a mesma convenção já aplicada às
demais figuras da análise: o título passa a viver apenas no nome do
arquivo e na legenda (caption) da tese. Mantém os rótulos dos painéis
por período (2020-2021, 2022-2023, 2024), análogos aos rótulos de grupo
preservados na figura 7. Regenera as figuras em output/coword/ e figuras/.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YJkP9yG5LdjoMqyurkKK9A
</commit_message>
<xml_diff>
--- a/output/coword/coword_nos_comunidades.xlsx
+++ b/output/coword/coword_nos_comunidades.xlsx
@@ -537,7 +537,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>dynamic</t>
+          <t>ocean</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -547,13 +547,13 @@
         <v>0</v>
       </c>
       <c r="D8" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ocean</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -563,7 +563,7 @@
         <v>0</v>
       </c>
       <c r="D9" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="10">
@@ -617,7 +617,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>state</t>
+          <t>graph neural</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -627,13 +627,13 @@
         <v>0</v>
       </c>
       <c r="D13" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>surface</t>
+          <t>state</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -643,13 +643,13 @@
         <v>0</v>
       </c>
       <c r="D14" t="n">
-        <v>15</v>
+        <v>7</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>graph neural</t>
+          <t>engineering</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -659,13 +659,13 @@
         <v>0</v>
       </c>
       <c r="D15" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>engineering</t>
+          <t>surface</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -675,7 +675,7 @@
         <v>0</v>
       </c>
       <c r="D16" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
     </row>
     <row r="17">
@@ -697,7 +697,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>textual</t>
+          <t>estimation</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -713,7 +713,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>offshore</t>
+          <t>physics-informed</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -723,7 +723,7 @@
         <v>0</v>
       </c>
       <c r="D19" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="20">
@@ -745,7 +745,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>resilience</t>
+          <t>physics-informed neural</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -761,7 +761,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>selection</t>
+          <t>offshore</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -771,13 +771,13 @@
         <v>0</v>
       </c>
       <c r="D22" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>physics-informed</t>
+          <t>propagation</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -787,13 +787,13 @@
         <v>0</v>
       </c>
       <c r="D23" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>estimation</t>
+          <t>assessment</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -803,13 +803,13 @@
         <v>0</v>
       </c>
       <c r="D24" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>physics-informed neural</t>
+          <t>resilience</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -825,7 +825,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>assessment</t>
+          <t>selection</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -835,13 +835,13 @@
         <v>0</v>
       </c>
       <c r="D26" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>propagation</t>
+          <t>textual</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -851,13 +851,13 @@
         <v>0</v>
       </c>
       <c r="D27" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>echo state</t>
+          <t>synchronization</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -867,13 +867,13 @@
         <v>0</v>
       </c>
       <c r="D28" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>insurance</t>
+          <t>event</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -883,13 +883,13 @@
         <v>0</v>
       </c>
       <c r="D29" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>operator</t>
+          <t>neural operator</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -905,7 +905,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>event</t>
+          <t>ocean offshore</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -915,13 +915,13 @@
         <v>0</v>
       </c>
       <c r="D31" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>synchronization</t>
+          <t>fine-tuning</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -931,13 +931,13 @@
         <v>0</v>
       </c>
       <c r="D32" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>state networks</t>
+          <t>joint</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -953,7 +953,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>bayesian</t>
+          <t>state networks</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -963,13 +963,13 @@
         <v>0</v>
       </c>
       <c r="D34" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>forecasting</t>
+          <t>semi-supervised</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -979,13 +979,13 @@
         <v>0</v>
       </c>
       <c r="D35" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>feature</t>
+          <t>forecasting</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -995,13 +995,13 @@
         <v>0</v>
       </c>
       <c r="D36" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>semi-supervised</t>
+          <t>bayesian</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1011,13 +1011,13 @@
         <v>0</v>
       </c>
       <c r="D37" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>joint</t>
+          <t>operator</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1033,7 +1033,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>echo</t>
+          <t>feature</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1043,13 +1043,13 @@
         <v>0</v>
       </c>
       <c r="D39" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>ocean offshore</t>
+          <t>echo</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1059,13 +1059,13 @@
         <v>0</v>
       </c>
       <c r="D40" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>fine-tuning</t>
+          <t>echo state</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1075,119 +1075,119 @@
         <v>0</v>
       </c>
       <c r="D41" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>index</t>
+          <t>data</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>4</v>
+        <v>38</v>
       </c>
       <c r="C42" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D42" t="n">
-        <v>5</v>
+        <v>56</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>neural operator</t>
+          <t>artificial</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>4</v>
+        <v>31</v>
       </c>
       <c r="C43" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D43" t="n">
-        <v>7</v>
+        <v>23</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>data</t>
+          <t>intelligence</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>38</v>
+        <v>19</v>
       </c>
       <c r="C44" t="n">
         <v>1</v>
       </c>
       <c r="D44" t="n">
-        <v>56</v>
+        <v>27</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>artificial</t>
+          <t>artificial intelligence</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>31</v>
+        <v>15</v>
       </c>
       <c r="C45" t="n">
         <v>1</v>
       </c>
       <c r="D45" t="n">
-        <v>23</v>
+        <v>16</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>intelligence</t>
+          <t>detection</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="C46" t="n">
         <v>1</v>
       </c>
       <c r="D46" t="n">
-        <v>27</v>
+        <v>21</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>artificial intelligence</t>
+          <t>optimization</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C47" t="n">
         <v>1</v>
       </c>
       <c r="D47" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>detection</t>
+          <t>inteligência artificial</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C48" t="n">
         <v>1</v>
       </c>
       <c r="D48" t="n">
-        <v>21</v>
+        <v>3</v>
       </c>
     </row>
     <row r="49">
@@ -1209,139 +1209,139 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>inteligência artificial</t>
+          <t>processing</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="C50" t="n">
         <v>1</v>
       </c>
       <c r="D50" t="n">
-        <v>3</v>
+        <v>21</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>optimization</t>
+          <t>news</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="C51" t="n">
         <v>1</v>
       </c>
       <c r="D51" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>datasets</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="C52" t="n">
         <v>1</v>
       </c>
       <c r="D52" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>news</t>
+          <t>multimodal</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C53" t="n">
         <v>1</v>
       </c>
       <c r="D53" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>fair</t>
+          <t>agricultural</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C54" t="n">
         <v>1</v>
       </c>
       <c r="D54" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>opinion</t>
+          <t>applied</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C55" t="n">
         <v>1</v>
       </c>
       <c r="D55" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>datasets</t>
+          <t>data augmentation</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C56" t="n">
         <v>1</v>
       </c>
       <c r="D56" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>multimodal</t>
+          <t>augmentation</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C57" t="n">
         <v>1</v>
       </c>
       <c r="D57" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>agricultural</t>
+          <t>fake</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C58" t="n">
         <v>1</v>
@@ -1369,7 +1369,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>set</t>
+          <t>fake news</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -1385,7 +1385,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>fake news</t>
+          <t>mining</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -1395,109 +1395,109 @@
         <v>1</v>
       </c>
       <c r="D61" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>applied</t>
+          <t>knowledge</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C62" t="n">
         <v>1</v>
       </c>
       <c r="D62" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>mining</t>
+          <t>amazon</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C63" t="n">
         <v>1</v>
       </c>
       <c r="D63" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>agriculture</t>
+          <t>early</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C64" t="n">
         <v>1</v>
       </c>
       <c r="D64" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>data augmentation</t>
+          <t>build</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C65" t="n">
         <v>1</v>
       </c>
       <c r="D65" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>fake</t>
+          <t>extrusion</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C66" t="n">
         <v>1</v>
       </c>
       <c r="D66" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>augmentation</t>
+          <t>multi-objective</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C67" t="n">
         <v>1</v>
       </c>
       <c r="D67" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>extrusion</t>
+          <t>data intelligence</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -1507,13 +1507,13 @@
         <v>1</v>
       </c>
       <c r="D68" t="n">
-        <v>6</v>
+        <v>14</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>facial</t>
+          <t>blue amazon</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -1523,13 +1523,13 @@
         <v>1</v>
       </c>
       <c r="D69" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>build</t>
+          <t>blue</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -1539,7 +1539,7 @@
         <v>1</v>
       </c>
       <c r="D70" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="71">
@@ -1561,7 +1561,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>building</t>
+          <t>low-resource</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -1571,13 +1571,13 @@
         <v>1</v>
       </c>
       <c r="D72" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>knowledge</t>
+          <t>algorithms</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -1587,13 +1587,13 @@
         <v>1</v>
       </c>
       <c r="D73" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>blue</t>
+          <t>facial</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -1603,493 +1603,493 @@
         <v>1</v>
       </c>
       <c r="D74" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>algorithms</t>
+          <t>brazilian</t>
         </is>
       </c>
       <c r="B75" t="n">
-        <v>4</v>
+        <v>53</v>
       </c>
       <c r="C75" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D75" t="n">
-        <v>1</v>
+        <v>66</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>low-resource</t>
+          <t>portuguese</t>
         </is>
       </c>
       <c r="B76" t="n">
-        <v>4</v>
+        <v>50</v>
       </c>
       <c r="C76" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D76" t="n">
-        <v>4</v>
+        <v>50</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>amazon</t>
+          <t>speech</t>
         </is>
       </c>
       <c r="B77" t="n">
-        <v>4</v>
+        <v>22</v>
       </c>
       <c r="C77" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D77" t="n">
-        <v>8</v>
+        <v>35</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>data intelligence</t>
+          <t>language</t>
         </is>
       </c>
       <c r="B78" t="n">
-        <v>4</v>
+        <v>21</v>
       </c>
       <c r="C78" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D78" t="n">
-        <v>14</v>
+        <v>26</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>blue amazon</t>
+          <t>brazilian portuguese</t>
         </is>
       </c>
       <c r="B79" t="n">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="C79" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D79" t="n">
-        <v>8</v>
+        <v>22</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>early</t>
+          <t>corpus</t>
         </is>
       </c>
       <c r="B80" t="n">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="C80" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D80" t="n">
-        <v>8</v>
+        <v>28</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>multi-objective</t>
+          <t>evaluation</t>
         </is>
       </c>
       <c r="B81" t="n">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="C81" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D81" t="n">
-        <v>3</v>
+        <v>25</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>brazilian</t>
+          <t>recognition</t>
         </is>
       </c>
       <c r="B82" t="n">
-        <v>53</v>
+        <v>14</v>
       </c>
       <c r="C82" t="n">
         <v>2</v>
       </c>
       <c r="D82" t="n">
-        <v>66</v>
+        <v>23</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>portuguese</t>
+          <t>intelligent</t>
         </is>
       </c>
       <c r="B83" t="n">
-        <v>50</v>
+        <v>13</v>
       </c>
       <c r="C83" t="n">
         <v>2</v>
       </c>
       <c r="D83" t="n">
-        <v>50</v>
+        <v>11</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>speech</t>
+          <t>automatic</t>
         </is>
       </c>
       <c r="B84" t="n">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="C84" t="n">
         <v>2</v>
       </c>
       <c r="D84" t="n">
-        <v>35</v>
+        <v>8</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>language</t>
+          <t>resources</t>
         </is>
       </c>
       <c r="B85" t="n">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="C85" t="n">
         <v>2</v>
       </c>
       <c r="D85" t="n">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>brazilian portuguese</t>
+          <t>bracis</t>
         </is>
       </c>
       <c r="B86" t="n">
-        <v>19</v>
+        <v>7</v>
       </c>
       <c r="C86" t="n">
         <v>2</v>
       </c>
       <c r="D86" t="n">
-        <v>22</v>
+        <v>4</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>corpus</t>
+          <t>speech recognition</t>
         </is>
       </c>
       <c r="B87" t="n">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="C87" t="n">
         <v>2</v>
       </c>
       <c r="D87" t="n">
-        <v>28</v>
+        <v>13</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>evaluation</t>
+          <t>spontaneous</t>
         </is>
       </c>
       <c r="B88" t="n">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="C88" t="n">
         <v>2</v>
       </c>
       <c r="D88" t="n">
-        <v>25</v>
+        <v>13</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>recognition</t>
+          <t>asr</t>
         </is>
       </c>
       <c r="B89" t="n">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="C89" t="n">
         <v>2</v>
       </c>
       <c r="D89" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>intelligent</t>
+          <t>public</t>
         </is>
       </c>
       <c r="B90" t="n">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="C90" t="n">
         <v>2</v>
       </c>
       <c r="D90" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>automatic</t>
+          <t>design</t>
         </is>
       </c>
       <c r="B91" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="C91" t="n">
         <v>2</v>
       </c>
       <c r="D91" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>processing</t>
+          <t>cham</t>
         </is>
       </c>
       <c r="B92" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="C92" t="n">
         <v>2</v>
       </c>
       <c r="D92" t="n">
-        <v>21</v>
+        <v>3</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>resources</t>
+          <t>portuguese language</t>
         </is>
       </c>
       <c r="B93" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="C93" t="n">
         <v>2</v>
       </c>
       <c r="D93" t="n">
-        <v>24</v>
+        <v>8</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>natural</t>
+          <t>extraction</t>
         </is>
       </c>
       <c r="B94" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C94" t="n">
         <v>2</v>
       </c>
       <c r="D94" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>bracis</t>
+          <t>emotion</t>
         </is>
       </c>
       <c r="B95" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C95" t="n">
         <v>2</v>
       </c>
       <c r="D95" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>asr</t>
+          <t>insurance</t>
         </is>
       </c>
       <c r="B96" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C96" t="n">
         <v>2</v>
       </c>
       <c r="D96" t="n">
-        <v>19</v>
+        <v>4</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>spontaneous</t>
+          <t>manually</t>
         </is>
       </c>
       <c r="B97" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C97" t="n">
         <v>2</v>
       </c>
       <c r="D97" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>public</t>
+          <t>coraa</t>
         </is>
       </c>
       <c r="B98" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C98" t="n">
         <v>2</v>
       </c>
       <c r="D98" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>speech recognition</t>
+          <t>corpora</t>
         </is>
       </c>
       <c r="B99" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C99" t="n">
         <v>2</v>
       </c>
       <c r="D99" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>cham</t>
+          <t>features</t>
         </is>
       </c>
       <c r="B100" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C100" t="n">
         <v>2</v>
       </c>
       <c r="D100" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>design</t>
+          <t>latin</t>
         </is>
       </c>
       <c r="B101" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C101" t="n">
         <v>2</v>
       </c>
       <c r="D101" t="n">
-        <v>13</v>
+        <v>3</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>extraction</t>
+          <t>spoken</t>
         </is>
       </c>
       <c r="B102" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C102" t="n">
         <v>2</v>
       </c>
       <c r="D102" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>portuguese language</t>
+          <t>index</t>
         </is>
       </c>
       <c r="B103" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C103" t="n">
         <v>2</v>
       </c>
       <c r="D103" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>natural language</t>
+          <t>development</t>
         </is>
       </c>
       <c r="B104" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C104" t="n">
         <v>2</v>
       </c>
       <c r="D104" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>formal</t>
+          <t>online</t>
         </is>
       </c>
       <c r="B105" t="n">
@@ -2099,13 +2099,13 @@
         <v>2</v>
       </c>
       <c r="D105" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>manually</t>
+          <t>emotion recognition</t>
         </is>
       </c>
       <c r="B106" t="n">
@@ -2115,321 +2115,321 @@
         <v>2</v>
       </c>
       <c r="D106" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>emotion</t>
+          <t>languages</t>
         </is>
       </c>
       <c r="B107" t="n">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="C107" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D107" t="n">
-        <v>5</v>
+        <v>21</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>corpora</t>
+          <t>indigenous</t>
         </is>
       </c>
       <c r="B108" t="n">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="C108" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D108" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>coraa</t>
+          <t>indigenous languages</t>
         </is>
       </c>
       <c r="B109" t="n">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="C109" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D109" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>probabilistic</t>
+          <t>prediction</t>
         </is>
       </c>
       <c r="B110" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="C110" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D110" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>online</t>
+          <t>social</t>
         </is>
       </c>
       <c r="B111" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="C111" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D111" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>development</t>
+          <t>impact</t>
         </is>
       </c>
       <c r="B112" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C112" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D112" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>emotion recognition</t>
+          <t>ethical</t>
         </is>
       </c>
       <c r="B113" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C113" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D113" t="n">
-        <v>5</v>
+        <v>14</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>latin</t>
+          <t>training</t>
         </is>
       </c>
       <c r="B114" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C114" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D114" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>features</t>
+          <t>brazilian indigenous</t>
         </is>
       </c>
       <c r="B115" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C115" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D115" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>science</t>
+          <t>media</t>
         </is>
       </c>
       <c r="B116" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C116" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D116" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>computer</t>
+          <t>smart</t>
         </is>
       </c>
       <c r="B117" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C117" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D117" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>spoken</t>
+          <t>identification</t>
         </is>
       </c>
       <c r="B118" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C118" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D118" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>universal</t>
+          <t>social media</t>
         </is>
       </c>
       <c r="B119" t="n">
-        <v>32</v>
+        <v>5</v>
       </c>
       <c r="C119" t="n">
         <v>3</v>
       </c>
       <c r="D119" t="n">
-        <v>23</v>
+        <v>4</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>dependencies</t>
+          <t>evaluating</t>
         </is>
       </c>
       <c r="B120" t="n">
-        <v>31</v>
+        <v>5</v>
       </c>
       <c r="C120" t="n">
         <v>3</v>
       </c>
       <c r="D120" t="n">
-        <v>24</v>
+        <v>4</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>universal dependencies</t>
+          <t>endangered</t>
         </is>
       </c>
       <c r="B121" t="n">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="C121" t="n">
         <v>3</v>
       </c>
       <c r="D121" t="n">
-        <v>23</v>
+        <v>7</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>português</t>
+          <t>good</t>
         </is>
       </c>
       <c r="B122" t="n">
-        <v>23</v>
+        <v>4</v>
       </c>
       <c r="C122" t="n">
         <v>3</v>
       </c>
       <c r="D122" t="n">
-        <v>27</v>
+        <v>11</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>brasileiro</t>
+          <t>research</t>
         </is>
       </c>
       <c r="B123" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="C123" t="n">
         <v>3</v>
       </c>
       <c r="D123" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>dados</t>
+          <t>toy</t>
         </is>
       </c>
       <c r="B124" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C124" t="n">
         <v>3</v>
       </c>
       <c r="D124" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>september</t>
+          <t>articles</t>
         </is>
       </c>
       <c r="B125" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C125" t="n">
         <v>3</v>
       </c>
       <c r="D125" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>tweets</t>
+          <t>constraints</t>
         </is>
       </c>
       <c r="B126" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C126" t="n">
         <v>3</v>
@@ -2441,238 +2441,238 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>texts</t>
+          <t>community</t>
         </is>
       </c>
       <c r="B127" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C127" t="n">
         <v>3</v>
       </c>
       <c r="D127" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>brasil</t>
+          <t>exploratory</t>
         </is>
       </c>
       <c r="B128" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C128" t="n">
         <v>3</v>
       </c>
       <c r="D128" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>portugues</t>
+          <t>human</t>
         </is>
       </c>
       <c r="B129" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C129" t="n">
         <v>3</v>
       </c>
       <c r="D129" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>estudo</t>
+          <t>smart toy</t>
         </is>
       </c>
       <c r="B130" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C130" t="n">
         <v>3</v>
       </c>
       <c r="D130" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>lexical</t>
+          <t>universal</t>
         </is>
       </c>
       <c r="B131" t="n">
-        <v>6</v>
+        <v>32</v>
       </c>
       <c r="C131" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D131" t="n">
-        <v>4</v>
+        <v>23</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>mercado</t>
+          <t>dependencies</t>
         </is>
       </c>
       <c r="B132" t="n">
-        <v>6</v>
+        <v>31</v>
       </c>
       <c r="C132" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D132" t="n">
-        <v>6</v>
+        <v>24</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>parsing</t>
+          <t>universal dependencies</t>
         </is>
       </c>
       <c r="B133" t="n">
-        <v>6</v>
+        <v>29</v>
       </c>
       <c r="C133" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D133" t="n">
-        <v>10</v>
+        <v>23</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>mercado financeiro</t>
+          <t>português</t>
         </is>
       </c>
       <c r="B134" t="n">
-        <v>6</v>
+        <v>23</v>
       </c>
       <c r="C134" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D134" t="n">
-        <v>6</v>
+        <v>27</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>financeiro</t>
+          <t>brasileiro</t>
         </is>
       </c>
       <c r="B135" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="C135" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D135" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>construções</t>
+          <t>estudo</t>
         </is>
       </c>
       <c r="B136" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C136" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D136" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>annotation</t>
+          <t>september</t>
         </is>
       </c>
       <c r="B137" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C137" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D137" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>segundo</t>
+          <t>brasil</t>
         </is>
       </c>
       <c r="B138" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C138" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D138" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>análise</t>
+          <t>texts</t>
         </is>
       </c>
       <c r="B139" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C139" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D139" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>linguagem</t>
+          <t>portugues</t>
         </is>
       </c>
       <c r="B140" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C140" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D140" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>caso</t>
+          <t>construções</t>
         </is>
       </c>
       <c r="B141" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C141" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D141" t="n">
         <v>8</v>
@@ -2681,46 +2681,46 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>português brasileiro</t>
+          <t>parsing</t>
         </is>
       </c>
       <c r="B142" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C142" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D142" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>abralin</t>
+          <t>lexical</t>
         </is>
       </c>
       <c r="B143" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C143" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D143" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>portuguese texts</t>
+          <t>segundo</t>
         </is>
       </c>
       <c r="B144" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C144" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D144" t="n">
         <v>7</v>
@@ -2729,190 +2729,190 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>processamento</t>
+          <t>português brasileiro</t>
         </is>
       </c>
       <c r="B145" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C145" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D145" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>tweets mercado</t>
+          <t>annotation</t>
         </is>
       </c>
       <c r="B146" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C146" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D146" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>relações</t>
+          <t>linguagem</t>
         </is>
       </c>
       <c r="B147" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C147" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D147" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>annotated</t>
+          <t>análise</t>
         </is>
       </c>
       <c r="B148" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C148" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D148" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>informação</t>
+          <t>relações</t>
         </is>
       </c>
       <c r="B149" t="n">
         <v>4</v>
       </c>
       <c r="C149" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D149" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>languages</t>
+          <t>portuguese texts</t>
         </is>
       </c>
       <c r="B150" t="n">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="C150" t="n">
         <v>4</v>
       </c>
       <c r="D150" t="n">
-        <v>21</v>
+        <v>7</v>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>indigenous</t>
+          <t>annotated</t>
         </is>
       </c>
       <c r="B151" t="n">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="C151" t="n">
         <v>4</v>
       </c>
       <c r="D151" t="n">
-        <v>18</v>
+        <v>9</v>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>indigenous languages</t>
+          <t>processamento</t>
         </is>
       </c>
       <c r="B152" t="n">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="C152" t="n">
         <v>4</v>
       </c>
       <c r="D152" t="n">
-        <v>18</v>
+        <v>3</v>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>prediction</t>
+          <t>informação</t>
         </is>
       </c>
       <c r="B153" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="C153" t="n">
         <v>4</v>
       </c>
       <c r="D153" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>social</t>
+          <t>abralin</t>
         </is>
       </c>
       <c r="B154" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="C154" t="n">
         <v>4</v>
       </c>
       <c r="D154" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>impact</t>
+          <t>modeling</t>
         </is>
       </c>
       <c r="B155" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="C155" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D155" t="n">
-        <v>7</v>
+        <v>18</v>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>ethical</t>
+          <t>dataset</t>
         </is>
       </c>
       <c r="B156" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C156" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D156" t="n">
         <v>14</v>
@@ -2921,318 +2921,318 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>media</t>
+          <t>model</t>
         </is>
       </c>
       <c r="B157" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C157" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D157" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>training</t>
+          <t>climate</t>
         </is>
       </c>
       <c r="B158" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C158" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D158" t="n">
-        <v>5</v>
+        <v>16</v>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>brazilian indigenous</t>
+          <t>change</t>
         </is>
       </c>
       <c r="B159" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C159" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D159" t="n">
-        <v>9</v>
+        <v>18</v>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>smart</t>
+          <t>climate change</t>
         </is>
       </c>
       <c r="B160" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C160" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D160" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>evaluating</t>
+          <t>time</t>
         </is>
       </c>
       <c r="B161" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C161" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D161" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>identification</t>
+          <t>variables</t>
         </is>
       </c>
       <c r="B162" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C162" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D162" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>social media</t>
+          <t>tasks</t>
         </is>
       </c>
       <c r="B163" t="n">
         <v>5</v>
       </c>
       <c r="C163" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D163" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>human</t>
+          <t>chatgpt</t>
         </is>
       </c>
       <c r="B164" t="n">
         <v>4</v>
       </c>
       <c r="C164" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D164" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>toy</t>
+          <t>oceanic variables</t>
         </is>
       </c>
       <c r="B165" t="n">
         <v>4</v>
       </c>
       <c r="C165" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D165" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>constraints</t>
+          <t>assessing</t>
         </is>
       </c>
       <c r="B166" t="n">
         <v>4</v>
       </c>
       <c r="C166" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D166" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>research</t>
+          <t>series</t>
         </is>
       </c>
       <c r="B167" t="n">
         <v>4</v>
       </c>
       <c r="C167" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D167" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>community</t>
+          <t>oceanic</t>
         </is>
       </c>
       <c r="B168" t="n">
         <v>4</v>
       </c>
       <c r="C168" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D168" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>endangered</t>
+          <t>time series</t>
         </is>
       </c>
       <c r="B169" t="n">
         <v>4</v>
       </c>
       <c r="C169" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D169" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>exploratory</t>
+          <t>oceans</t>
         </is>
       </c>
       <c r="B170" t="n">
         <v>4</v>
       </c>
       <c r="C170" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D170" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>good</t>
+          <t>learning</t>
         </is>
       </c>
       <c r="B171" t="n">
-        <v>4</v>
+        <v>33</v>
       </c>
       <c r="C171" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D171" t="n">
-        <v>11</v>
+        <v>24</v>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>smart toy</t>
+          <t>models</t>
         </is>
       </c>
       <c r="B172" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="C172" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D172" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>articles</t>
+          <t>deep</t>
         </is>
       </c>
       <c r="B173" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="C173" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D173" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>modeling</t>
+          <t>machine learning</t>
         </is>
       </c>
       <c r="B174" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="C174" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D174" t="n">
-        <v>18</v>
+        <v>8</v>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>dataset</t>
+          <t>machine</t>
         </is>
       </c>
       <c r="B175" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C175" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D175" t="n">
-        <v>14</v>
+        <v>8</v>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>model</t>
+          <t>deep learning</t>
         </is>
       </c>
       <c r="B176" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C176" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D176" t="n">
         <v>6</v>
@@ -3241,318 +3241,318 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>climate</t>
+          <t>covid-</t>
         </is>
       </c>
       <c r="B177" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C177" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D177" t="n">
-        <v>16</v>
+        <v>5</v>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>change</t>
+          <t>segmentation</t>
         </is>
       </c>
       <c r="B178" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="C178" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D178" t="n">
-        <v>18</v>
+        <v>5</v>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>climate change</t>
+          <t>sentiment</t>
         </is>
       </c>
       <c r="B179" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C179" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D179" t="n">
-        <v>15</v>
+        <v>7</v>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>time</t>
+          <t>representation</t>
         </is>
       </c>
       <c r="B180" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C180" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D180" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>variables</t>
+          <t>benchmark</t>
         </is>
       </c>
       <c r="B181" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C181" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D181" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>tasks</t>
+          <t>semantic</t>
         </is>
       </c>
       <c r="B182" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C182" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D182" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>series</t>
+          <t>computational</t>
         </is>
       </c>
       <c r="B183" t="n">
         <v>4</v>
       </c>
       <c r="C183" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D183" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>oceanic</t>
+          <t>automated</t>
         </is>
       </c>
       <c r="B184" t="n">
         <v>4</v>
       </c>
       <c r="C184" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D184" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>chatgpt</t>
+          <t>patients</t>
         </is>
       </c>
       <c r="B185" t="n">
         <v>4</v>
       </c>
       <c r="C185" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D185" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>time series</t>
+          <t>dados</t>
         </is>
       </c>
       <c r="B186" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="C186" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D186" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>oceans</t>
+          <t>tweets</t>
         </is>
       </c>
       <c r="B187" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C187" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D187" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>oceanic variables</t>
+          <t>mercado financeiro</t>
         </is>
       </c>
       <c r="B188" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C188" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D188" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>assessing</t>
+          <t>financeiro</t>
         </is>
       </c>
       <c r="B189" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C189" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D189" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>learning</t>
+          <t>mercado</t>
         </is>
       </c>
       <c r="B190" t="n">
-        <v>33</v>
+        <v>6</v>
       </c>
       <c r="C190" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D190" t="n">
-        <v>24</v>
+        <v>6</v>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>models</t>
+          <t>caso</t>
         </is>
       </c>
       <c r="B191" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="C191" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D191" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>deep</t>
+          <t>tweets mercado</t>
         </is>
       </c>
       <c r="B192" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="C192" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D192" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>machine learning</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B193" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C193" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D193" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>machine</t>
+          <t>fair</t>
         </is>
       </c>
       <c r="B194" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C194" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D194" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>deep learning</t>
+          <t>opinion</t>
         </is>
       </c>
       <c r="B195" t="n">
+        <v>7</v>
+      </c>
+      <c r="C195" t="n">
         <v>8</v>
       </c>
-      <c r="C195" t="n">
-        <v>6</v>
-      </c>
       <c r="D195" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>covid-</t>
+          <t>set</t>
         </is>
       </c>
       <c r="B196" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C196" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D196" t="n">
         <v>5</v>
@@ -3561,14 +3561,14 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>segmentation</t>
+          <t>agriculture</t>
         </is>
       </c>
       <c r="B197" t="n">
         <v>5</v>
       </c>
       <c r="C197" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D197" t="n">
         <v>5</v>
@@ -3577,46 +3577,46 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>representation</t>
+          <t>building</t>
         </is>
       </c>
       <c r="B198" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C198" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D198" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>benchmark</t>
+          <t>natural</t>
         </is>
       </c>
       <c r="B199" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C199" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D199" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>sentiment</t>
+          <t>natural language</t>
         </is>
       </c>
       <c r="B200" t="n">
         <v>5</v>
       </c>
       <c r="C200" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D200" t="n">
         <v>7</v>
@@ -3625,65 +3625,65 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>computational</t>
+          <t>science</t>
         </is>
       </c>
       <c r="B201" t="n">
         <v>4</v>
       </c>
       <c r="C201" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D201" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>patients</t>
+          <t>formal</t>
         </is>
       </c>
       <c r="B202" t="n">
         <v>4</v>
       </c>
       <c r="C202" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D202" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>automated</t>
+          <t>probabilistic</t>
         </is>
       </c>
       <c r="B203" t="n">
         <v>4</v>
       </c>
       <c r="C203" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D203" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>semantic</t>
+          <t>computer</t>
         </is>
       </c>
       <c r="B204" t="n">
         <v>4</v>
       </c>
       <c r="C204" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D204" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="205">
@@ -3696,7 +3696,7 @@
         <v>4</v>
       </c>
       <c r="C205" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="D205" t="n">
         <v>1</v>
@@ -3712,7 +3712,7 @@
         <v>4</v>
       </c>
       <c r="C206" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="D206" t="n">
         <v>1</v>
@@ -3728,7 +3728,7 @@
         <v>6</v>
       </c>
       <c r="C207" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="D207" t="n">
         <v>1</v>
@@ -3744,7 +3744,7 @@
         <v>4</v>
       </c>
       <c r="C208" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="D208" t="n">
         <v>1</v>

</xml_diff>